<commit_message>
feat: l2 gap (#73)
</commit_message>
<xml_diff>
--- a/docs/samples/orbit-sample-l1-demo.xlsx
+++ b/docs/samples/orbit-sample-l1-demo.xlsx
@@ -94,6 +94,12 @@
     <x:t>DependsOn</x:t>
   </x:si>
   <x:si>
+    <x:t>BaselineDate</x:t>
+  </x:si>
+  <x:si>
+    <x:t>IsCritical</x:t>
+  </x:si>
+  <x:si>
     <x:t>POS pilot live</x:t>
   </x:si>
   <x:si>
@@ -106,6 +112,12 @@
     <x:t>In Progress</x:t>
   </x:si>
   <x:si>
+    <x:t>2026-07-15</x:t>
+  </x:si>
+  <x:si>
+    <x:t>true</x:t>
+  </x:si>
+  <x:si>
     <x:t>Data cutover dress rehearsal</x:t>
   </x:si>
   <x:si>
@@ -115,12 +127,18 @@
     <x:t>Missed</x:t>
   </x:si>
   <x:si>
+    <x:t>2026-05-30</x:t>
+  </x:si>
+  <x:si>
     <x:t>SCA remediation done</x:t>
   </x:si>
   <x:si>
     <x:t>2026-07-20</x:t>
   </x:si>
   <x:si>
+    <x:t>false</x:t>
+  </x:si>
+  <x:si>
     <x:t>Category</x:t>
   </x:si>
   <x:si>
@@ -196,9 +214,6 @@
     <x:t>100</x:t>
   </x:si>
   <x:si>
-    <x:t>false</x:t>
-  </x:si>
-  <x:si>
     <x:t>Jonas Vik</x:t>
   </x:si>
   <x:si>
@@ -290,9 +305,6 @@
   </x:si>
   <x:si>
     <x:t>Client Sponsor</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-07-15</x:t>
   </x:si>
   <x:si>
     <x:t>Integrity errors persist into production</x:t>
@@ -788,10 +800,10 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:F4"/>
+  <x:dimension ref="A1:H4"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
-    <x:row r="1" spans="1:6">
+    <x:row r="1" spans="1:8">
       <x:c r="A1" s="0" t="s">
         <x:v>19</x:v>
       </x:c>
@@ -810,65 +822,89 @@
       <x:c r="F1" s="0" t="s">
         <x:v>23</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2" spans="1:6">
+      <x:c r="G1" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="H1" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:8">
       <x:c r="A2" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>24</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>25</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>27</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>26</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:6">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="G2" s="0" t="s">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="H2" s="0" t="s">
+        <x:v>31</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:8">
       <x:c r="A3" s="0" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="C3" s="0" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="D3" s="0" t="s">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="C3" s="0" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="D3" s="0" t="s">
-        <x:v>26</x:v>
-      </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
-        <x:v>26</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:6">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="G3" s="0" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="H3" s="0" t="s">
+        <x:v>31</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:8">
       <x:c r="A4" s="0" t="s">
         <x:v>15</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>31</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>32</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>28</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>27</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="F4" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="G4" s="0" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="H4" s="0" t="s">
+        <x:v>38</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -893,19 +929,19 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>33</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>34</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>35</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>36</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>43</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:6">
@@ -913,19 +949,19 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>39</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>42</x:v>
+        <x:v>48</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:6">
@@ -933,19 +969,19 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>43</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>44</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>45</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
-        <x:v>42</x:v>
+        <x:v>48</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:6">
@@ -953,19 +989,19 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>46</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>47</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="F4" s="0" t="s">
         <x:v>48</x:v>
-      </x:c>
-      <x:c r="F4" s="0" t="s">
-        <x:v>42</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -990,19 +1026,19 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>51</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>52</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>59</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:6">
@@ -1010,19 +1046,19 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>55</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>56</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>58</x:v>
+        <x:v>38</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:6">
@@ -1030,19 +1066,19 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>59</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>60</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
-        <x:v>58</x:v>
+        <x:v>38</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:6">
@@ -1050,19 +1086,19 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>62</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>60</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="F4" s="0" t="s">
-        <x:v>58</x:v>
+        <x:v>38</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:6">
@@ -1070,19 +1106,19 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>55</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="E5" s="0" t="s">
         <x:v>63</x:v>
       </x:c>
-      <x:c r="E5" s="0" t="s">
-        <x:v>57</x:v>
-      </x:c>
       <x:c r="F5" s="0" t="s">
-        <x:v>58</x:v>
+        <x:v>38</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:6">
@@ -1090,19 +1126,19 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
-        <x:v>64</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
-        <x:v>60</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="E6" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="F6" s="0" t="s">
-        <x:v>58</x:v>
+        <x:v>38</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:6">
@@ -1110,19 +1146,19 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C7" s="0" t="s">
-        <x:v>55</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="D7" s="0" t="s">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="E7" s="0" t="s">
         <x:v>63</x:v>
       </x:c>
-      <x:c r="E7" s="0" t="s">
-        <x:v>57</x:v>
-      </x:c>
       <x:c r="F7" s="0" t="s">
-        <x:v>58</x:v>
+        <x:v>38</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:6">
@@ -1130,19 +1166,19 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B8" s="0" t="s">
-        <x:v>62</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C8" s="0" t="s">
-        <x:v>60</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="D8" s="0" t="s">
-        <x:v>65</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="E8" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="F8" s="0" t="s">
-        <x:v>58</x:v>
+        <x:v>38</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1167,13 +1203,13 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>66</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
         <x:v>22</x:v>
@@ -1184,16 +1220,16 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>69</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>70</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>72</x:v>
+        <x:v>77</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:5">
@@ -1201,16 +1237,16 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>69</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>73</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>74</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>72</x:v>
+        <x:v>77</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:5">
@@ -1218,16 +1254,16 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>75</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>76</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="E4" s="0" t="s">
         <x:v>77</x:v>
-      </x:c>
-      <x:c r="E4" s="0" t="s">
-        <x:v>72</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1252,19 +1288,19 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>78</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>80</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>81</x:v>
+        <x:v>86</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:6">
@@ -1272,19 +1308,19 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>82</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>83</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>84</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>85</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>86</x:v>
+        <x:v>91</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:6">
@@ -1292,19 +1328,19 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>87</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>88</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>89</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>90</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
-        <x:v>91</x:v>
+        <x:v>95</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:6">
@@ -1312,19 +1348,19 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>92</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>88</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>59</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>32</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="F4" s="0" t="s">
-        <x:v>93</x:v>
+        <x:v>97</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:6">
@@ -1332,19 +1368,19 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
-        <x:v>94</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>95</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="E5" s="0" t="s">
-        <x:v>96</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="F5" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>28</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1369,19 +1405,19 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>78</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>66</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>97</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>98</x:v>
+        <x:v>102</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:6">
@@ -1389,19 +1425,19 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>99</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>100</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>102</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>103</x:v>
+        <x:v>107</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:6">
@@ -1409,19 +1445,19 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
+        <x:v>108</x:v>
+      </x:c>
+      <x:c r="C3" s="0" t="s">
         <x:v>104</x:v>
       </x:c>
-      <x:c r="C3" s="0" t="s">
-        <x:v>100</x:v>
-      </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>95</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>105</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
-        <x:v>106</x:v>
+        <x:v>110</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:6">
@@ -1429,19 +1465,19 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>107</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>108</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>109</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="F4" s="0" t="s">
-        <x:v>110</x:v>
+        <x:v>114</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat: age column, suggested-remediation
</commit_message>
<xml_diff>
--- a/docs/samples/orbit-sample-l1-demo.xlsx
+++ b/docs/samples/orbit-sample-l1-demo.xlsx
@@ -79,6 +79,15 @@
     <x:t>2026-06-10</x:t>
   </x:si>
   <x:si>
+    <x:t>ORB-1002a</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Customer Data Migration Phase 2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>15</x:t>
+  </x:si>
+  <x:si>
     <x:t>ProjectKey</x:t>
   </x:si>
   <x:si>
@@ -187,6 +196,15 @@
     <x:t>470000</x:t>
   </x:si>
   <x:si>
+    <x:t>200000</x:t>
+  </x:si>
+  <x:si>
+    <x:t>210000</x:t>
+  </x:si>
+  <x:si>
+    <x:t>90000</x:t>
+  </x:si>
+  <x:si>
     <x:t>Person</x:t>
   </x:si>
   <x:si>
@@ -235,6 +253,9 @@
     <x:t>50</x:t>
   </x:si>
   <x:si>
+    <x:t>10</x:t>
+  </x:si>
+  <x:si>
     <x:t>Type</x:t>
   </x:si>
   <x:si>
@@ -347,9 +368,6 @@
   </x:si>
   <x:si>
     <x:t>Add loyalty module</x:t>
-  </x:si>
-  <x:si>
-    <x:t>10</x:t>
   </x:si>
   <x:si>
     <x:t>2026-06-01</x:t>
@@ -715,7 +733,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:E4"/>
+  <x:dimension ref="A1:E5"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:5">
@@ -783,6 +801,23 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:5">
+      <x:c r="A5" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D5" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="E5" s="0" t="s">
         <x:v>14</x:v>
       </x:c>
     </x:row>
@@ -805,28 +840,28 @@
   <x:sheetData>
     <x:row r="1" spans="1:8">
       <x:c r="A1" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
         <x:v>1</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>21</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="G1" s="0" t="s">
-        <x:v>24</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="H1" s="0" t="s">
-        <x:v>25</x:v>
+        <x:v>28</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:8">
@@ -834,25 +869,25 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>27</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="G2" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="H2" s="0" t="s">
-        <x:v>31</x:v>
+        <x:v>34</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:8">
@@ -860,25 +895,25 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>32</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>33</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="F3" s="0" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="G3" s="0" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="H3" s="0" t="s">
         <x:v>34</x:v>
-      </x:c>
-      <x:c r="F3" s="0" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="G3" s="0" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="H3" s="0" t="s">
-        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:8">
@@ -886,25 +921,25 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>36</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="F4" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="G4" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="H4" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>41</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -921,27 +956,27 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:F4"/>
+  <x:dimension ref="A1:F5"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:6">
       <x:c r="A1" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>42</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>43</x:v>
+        <x:v>46</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:6">
@@ -949,19 +984,19 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>44</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>45</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>46</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>47</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>48</x:v>
+        <x:v>51</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:6">
@@ -969,19 +1004,19 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>44</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="F3" s="0" t="s">
         <x:v>51</x:v>
-      </x:c>
-      <x:c r="F3" s="0" t="s">
-        <x:v>48</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:6">
@@ -989,19 +1024,39 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>44</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>52</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="F4" s="0" t="s">
-        <x:v>48</x:v>
+        <x:v>51</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:6">
+      <x:c r="A5" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="D5" s="0" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="E5" s="0" t="s">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="F5" s="0" t="s">
+        <x:v>51</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1018,27 +1073,27 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:F8"/>
+  <x:dimension ref="A1:F9"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:6">
       <x:c r="A1" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>55</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>56</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>58</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>59</x:v>
+        <x:v>65</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:6">
@@ -1046,19 +1101,19 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>60</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>62</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>41</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:6">
@@ -1066,19 +1121,19 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>64</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>65</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>66</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>41</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:6">
@@ -1086,19 +1141,19 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>65</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="F4" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>41</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:6">
@@ -1106,19 +1161,19 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
-        <x:v>60</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="E5" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="F5" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>41</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:6">
@@ -1126,19 +1181,19 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="C6" s="0" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="D6" s="0" t="s">
         <x:v>69</x:v>
       </x:c>
-      <x:c r="C6" s="0" t="s">
-        <x:v>65</x:v>
-      </x:c>
-      <x:c r="D6" s="0" t="s">
-        <x:v>63</x:v>
-      </x:c>
       <x:c r="E6" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="F6" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>41</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:6">
@@ -1146,19 +1201,19 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
-        <x:v>60</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="C7" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="D7" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="E7" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="F7" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>41</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:6">
@@ -1166,19 +1221,39 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B8" s="0" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="C8" s="0" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="D8" s="0" t="s">
+        <x:v>76</x:v>
+      </x:c>
+      <x:c r="E8" s="0" t="s">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="F8" s="0" t="s">
+        <x:v>41</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:6">
+      <x:c r="A9" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B9" s="0" t="s">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="C9" s="0" t="s">
         <x:v>67</x:v>
       </x:c>
-      <x:c r="C8" s="0" t="s">
-        <x:v>65</x:v>
-      </x:c>
-      <x:c r="D8" s="0" t="s">
-        <x:v>70</x:v>
-      </x:c>
-      <x:c r="E8" s="0" t="s">
-        <x:v>63</x:v>
-      </x:c>
-      <x:c r="F8" s="0" t="s">
-        <x:v>38</x:v>
+      <x:c r="D9" s="0" t="s">
+        <x:v>77</x:v>
+      </x:c>
+      <x:c r="E9" s="0" t="s">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="F9" s="0" t="s">
+        <x:v>41</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1200,19 +1275,19 @@
   <x:sheetData>
     <x:row r="1" spans="1:5">
       <x:c r="A1" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>72</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>73</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>25</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:5">
@@ -1220,16 +1295,16 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>74</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>75</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>76</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>77</x:v>
+        <x:v>84</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:5">
@@ -1237,16 +1312,16 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>74</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>78</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>77</x:v>
+        <x:v>84</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:5">
@@ -1254,16 +1329,16 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>80</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>81</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>82</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>77</x:v>
+        <x:v>84</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1285,22 +1360,22 @@
   <x:sheetData>
     <x:row r="1" spans="1:6">
       <x:c r="A1" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>83</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>84</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>85</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>86</x:v>
+        <x:v>93</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:6">
@@ -1308,19 +1383,19 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>87</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>88</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>89</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>90</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>91</x:v>
+        <x:v>98</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:6">
@@ -1328,19 +1403,19 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>92</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>93</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>94</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
-        <x:v>95</x:v>
+        <x:v>102</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:6">
@@ -1348,19 +1423,19 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>96</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>93</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>64</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="F4" s="0" t="s">
-        <x:v>97</x:v>
+        <x:v>104</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:6">
@@ -1368,19 +1443,19 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
-        <x:v>98</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>99</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>60</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="E5" s="0" t="s">
-        <x:v>100</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="F5" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>31</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1402,22 +1477,22 @@
   <x:sheetData>
     <x:row r="1" spans="1:6">
       <x:c r="A1" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>83</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>102</x:v>
+        <x:v>109</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:6">
@@ -1425,19 +1500,19 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>103</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>104</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>105</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>106</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>107</x:v>
+        <x:v>114</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:6">
@@ -1445,19 +1520,19 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>108</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>104</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>99</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>109</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
-        <x:v>110</x:v>
+        <x:v>116</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:6">
@@ -1465,19 +1540,19 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>111</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
+        <x:v>118</x:v>
+      </x:c>
+      <x:c r="D4" s="0" t="s">
         <x:v>112</x:v>
       </x:c>
-      <x:c r="D4" s="0" t="s">
-        <x:v>105</x:v>
-      </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>113</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="F4" s="0" t="s">
-        <x:v>114</x:v>
+        <x:v>120</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat: confidence and aread completeness
</commit_message>
<xml_diff>
--- a/docs/samples/orbit-sample-l1-demo.xlsx
+++ b/docs/samples/orbit-sample-l1-demo.xlsx
@@ -205,6 +205,12 @@
     <x:t>90000</x:t>
   </x:si>
   <x:si>
+    <x:t>Contingency</x:t>
+  </x:si>
+  <x:si>
+    <x:t>50000</x:t>
+  </x:si>
+  <x:si>
     <x:t>Person</x:t>
   </x:si>
   <x:si>
@@ -277,12 +283,18 @@
     <x:t>Open</x:t>
   </x:si>
   <x:si>
+    <x:t>2026-05-20</x:t>
+  </x:si>
+  <x:si>
     <x:t>POS vendor API rate limits block rollout</x:t>
   </x:si>
   <x:si>
     <x:t>High</x:t>
   </x:si>
   <x:si>
+    <x:t>2026-07-05</x:t>
+  </x:si>
+  <x:si>
     <x:t>Issue</x:t>
   </x:si>
   <x:si>
@@ -292,6 +304,9 @@
     <x:t>Medium</x:t>
   </x:si>
   <x:si>
+    <x:t>2026-06-01</x:t>
+  </x:si>
+  <x:si>
     <x:t>Title</x:t>
   </x:si>
   <x:si>
@@ -364,13 +379,7 @@
     <x:t>18</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-07-05</x:t>
-  </x:si>
-  <x:si>
     <x:t>Add loyalty module</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-06-01</x:t>
   </x:si>
   <x:si>
     <x:t>Drop legacy report export</x:t>
@@ -956,7 +965,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:F5"/>
+  <x:dimension ref="A1:F6"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:6">
@@ -1056,6 +1065,26 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="F5" s="0" t="s">
+        <x:v>51</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:6">
+      <x:c r="A6" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B6" s="0" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="C6" s="0" t="s">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="D6" s="0" t="s">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="E6" s="0" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="F6" s="0" t="s">
         <x:v>51</x:v>
       </x:c>
     </x:row>
@@ -1081,19 +1110,19 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>62</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>64</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>65</x:v>
+        <x:v>67</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:6">
@@ -1101,16 +1130,16 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>66</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>69</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
         <x:v>41</x:v>
@@ -1121,16 +1150,16 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>70</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="D3" s="0" t="s">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="E3" s="0" t="s">
         <x:v>71</x:v>
-      </x:c>
-      <x:c r="D3" s="0" t="s">
-        <x:v>72</x:v>
-      </x:c>
-      <x:c r="E3" s="0" t="s">
-        <x:v>69</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
         <x:v>41</x:v>
@@ -1141,16 +1170,16 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="s">
         <x:v>73</x:v>
       </x:c>
-      <x:c r="C4" s="0" t="s">
+      <x:c r="D4" s="0" t="s">
         <x:v>71</x:v>
       </x:c>
-      <x:c r="D4" s="0" t="s">
-        <x:v>69</x:v>
-      </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>69</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="F4" s="0" t="s">
         <x:v>41</x:v>
@@ -1161,16 +1190,16 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
-        <x:v>66</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>74</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="E5" s="0" t="s">
-        <x:v>69</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="F5" s="0" t="s">
         <x:v>41</x:v>
@@ -1181,16 +1210,16 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
-        <x:v>75</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="D6" s="0" t="s">
         <x:v>71</x:v>
       </x:c>
-      <x:c r="D6" s="0" t="s">
-        <x:v>69</x:v>
-      </x:c>
       <x:c r="E6" s="0" t="s">
-        <x:v>69</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="F6" s="0" t="s">
         <x:v>41</x:v>
@@ -1201,16 +1230,16 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
-        <x:v>66</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="C7" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="D7" s="0" t="s">
-        <x:v>74</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="E7" s="0" t="s">
-        <x:v>69</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="F7" s="0" t="s">
         <x:v>41</x:v>
@@ -1221,16 +1250,16 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B8" s="0" t="s">
+        <x:v>75</x:v>
+      </x:c>
+      <x:c r="C8" s="0" t="s">
         <x:v>73</x:v>
       </x:c>
-      <x:c r="C8" s="0" t="s">
+      <x:c r="D8" s="0" t="s">
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="E8" s="0" t="s">
         <x:v>71</x:v>
-      </x:c>
-      <x:c r="D8" s="0" t="s">
-        <x:v>76</x:v>
-      </x:c>
-      <x:c r="E8" s="0" t="s">
-        <x:v>69</x:v>
       </x:c>
       <x:c r="F8" s="0" t="s">
         <x:v>41</x:v>
@@ -1241,16 +1270,16 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="B9" s="0" t="s">
-        <x:v>66</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="C9" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="D9" s="0" t="s">
-        <x:v>77</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="E9" s="0" t="s">
-        <x:v>69</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="F9" s="0" t="s">
         <x:v>41</x:v>
@@ -1270,75 +1299,87 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:E4"/>
+  <x:dimension ref="A1:F4"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
-    <x:row r="1" spans="1:5">
+    <x:row r="1" spans="1:6">
       <x:c r="A1" s="0" t="s">
         <x:v>22</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>78</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>80</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
         <x:v>25</x:v>
       </x:c>
-    </x:row>
-    <x:row r="2" spans="1:5">
+      <x:c r="F1" s="0" t="s">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:6">
       <x:c r="A2" s="0" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>81</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>82</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>83</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>84</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:5">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="F2" s="0" t="s">
+        <x:v>87</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:6">
       <x:c r="A3" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>81</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>85</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
+        <x:v>89</x:v>
+      </x:c>
+      <x:c r="E3" s="0" t="s">
         <x:v>86</x:v>
       </x:c>
-      <x:c r="E3" s="0" t="s">
-        <x:v>84</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:5">
+      <x:c r="F3" s="0" t="s">
+        <x:v>90</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:6">
       <x:c r="A4" s="0" t="s">
         <x:v>15</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>87</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>88</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>89</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>84</x:v>
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="F4" s="0" t="s">
+        <x:v>94</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1363,19 +1404,19 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>90</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
         <x:v>25</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>91</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>92</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>93</x:v>
+        <x:v>98</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:6">
@@ -1383,19 +1424,19 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>94</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>95</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>96</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>97</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>98</x:v>
+        <x:v>103</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:6">
@@ -1403,19 +1444,19 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>99</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>100</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
         <x:v>33</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
-        <x:v>102</x:v>
+        <x:v>107</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:6">
@@ -1423,19 +1464,19 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>103</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>100</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>70</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
         <x:v>40</x:v>
       </x:c>
       <x:c r="F4" s="0" t="s">
-        <x:v>104</x:v>
+        <x:v>109</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:6">
@@ -1443,16 +1484,16 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
-        <x:v>105</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>106</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>66</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="E5" s="0" t="s">
-        <x:v>107</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="F5" s="0" t="s">
         <x:v>31</x:v>
@@ -1480,19 +1521,19 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>90</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>78</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
         <x:v>25</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>108</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>109</x:v>
+        <x:v>114</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:6">
@@ -1500,19 +1541,19 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>110</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>111</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>112</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>113</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>114</x:v>
+        <x:v>90</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:6">
@@ -1520,19 +1561,19 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>115</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
+        <x:v>116</x:v>
+      </x:c>
+      <x:c r="D3" s="0" t="s">
         <x:v>111</x:v>
       </x:c>
-      <x:c r="D3" s="0" t="s">
-        <x:v>106</x:v>
-      </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>77</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
-        <x:v>116</x:v>
+        <x:v>94</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:6">
@@ -1540,19 +1581,19 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="s">
+        <x:v>121</x:v>
+      </x:c>
+      <x:c r="D4" s="0" t="s">
         <x:v>117</x:v>
       </x:c>
-      <x:c r="C4" s="0" t="s">
-        <x:v>118</x:v>
-      </x:c>
-      <x:c r="D4" s="0" t="s">
-        <x:v>112</x:v>
-      </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>119</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="F4" s="0" t="s">
-        <x:v>120</x:v>
+        <x:v>123</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat: l3 gaps and update all documents (#74)
* feat: age column, suggested-remediation

* feat: confidence and aread completeness

* feat: data updated

* feat: add sample

* feat: update documents and code review

* feat: update doc

* feat: archirve add-decision-agent

* feat: archive add-finding-metric

* feat: archive add-structure-recommendation

* fix comment
</commit_message>
<xml_diff>
--- a/docs/samples/orbit-sample-l1-demo.xlsx
+++ b/docs/samples/orbit-sample-l1-demo.xlsx
@@ -13,6 +13,7 @@
     <x:sheet name="RAID" sheetId="5" r:id="rId6"/>
     <x:sheet name="Decisions" sheetId="6" r:id="rId7"/>
     <x:sheet name="Scope" sheetId="7" r:id="rId8"/>
+    <x:sheet name="Time" sheetId="8" r:id="rId9"/>
   </x:sheets>
   <x:definedNames/>
   <x:calcPr calcId="125725"/>
@@ -79,6 +80,15 @@
     <x:t>2026-06-10</x:t>
   </x:si>
   <x:si>
+    <x:t>ORB-1002a</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Customer Data Migration Phase 2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>15</x:t>
+  </x:si>
+  <x:si>
     <x:t>ProjectKey</x:t>
   </x:si>
   <x:si>
@@ -187,6 +197,21 @@
     <x:t>470000</x:t>
   </x:si>
   <x:si>
+    <x:t>200000</x:t>
+  </x:si>
+  <x:si>
+    <x:t>210000</x:t>
+  </x:si>
+  <x:si>
+    <x:t>90000</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Contingency</x:t>
+  </x:si>
+  <x:si>
+    <x:t>50000</x:t>
+  </x:si>
+  <x:si>
     <x:t>Person</x:t>
   </x:si>
   <x:si>
@@ -235,6 +260,9 @@
     <x:t>50</x:t>
   </x:si>
   <x:si>
+    <x:t>10</x:t>
+  </x:si>
+  <x:si>
     <x:t>Type</x:t>
   </x:si>
   <x:si>
@@ -256,12 +284,18 @@
     <x:t>Open</x:t>
   </x:si>
   <x:si>
+    <x:t>2026-05-20</x:t>
+  </x:si>
+  <x:si>
     <x:t>POS vendor API rate limits block rollout</x:t>
   </x:si>
   <x:si>
     <x:t>High</x:t>
   </x:si>
   <x:si>
+    <x:t>2026-07-05</x:t>
+  </x:si>
+  <x:si>
     <x:t>Issue</x:t>
   </x:si>
   <x:si>
@@ -271,6 +305,9 @@
     <x:t>Medium</x:t>
   </x:si>
   <x:si>
+    <x:t>2026-06-01</x:t>
+  </x:si>
+  <x:si>
     <x:t>Title</x:t>
   </x:si>
   <x:si>
@@ -343,18 +380,9 @@
     <x:t>18</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-07-05</x:t>
-  </x:si>
-  <x:si>
     <x:t>Add loyalty module</x:t>
   </x:si>
   <x:si>
-    <x:t>10</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2026-06-01</x:t>
-  </x:si>
-  <x:si>
     <x:t>Drop legacy report export</x:t>
   </x:si>
   <x:si>
@@ -365,6 +393,18 @@
   </x:si>
   <x:si>
     <x:t>2026-07-08</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HoursLogged</x:t>
+  </x:si>
+  <x:si>
+    <x:t>130</x:t>
+  </x:si>
+  <x:si>
+    <x:t>20</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Contractor X</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -715,7 +755,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:E4"/>
+  <x:dimension ref="A1:E5"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:5">
@@ -783,6 +823,23 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:5">
+      <x:c r="A5" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="D5" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="E5" s="0" t="s">
         <x:v>14</x:v>
       </x:c>
     </x:row>
@@ -805,28 +862,28 @@
   <x:sheetData>
     <x:row r="1" spans="1:8">
       <x:c r="A1" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
         <x:v>1</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>21</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>23</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="G1" s="0" t="s">
-        <x:v>24</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="H1" s="0" t="s">
-        <x:v>25</x:v>
+        <x:v>28</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:8">
@@ -834,25 +891,25 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>26</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>27</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="G2" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="H2" s="0" t="s">
-        <x:v>31</x:v>
+        <x:v>34</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:8">
@@ -860,25 +917,25 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>32</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>33</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="F3" s="0" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="G3" s="0" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="H3" s="0" t="s">
         <x:v>34</x:v>
-      </x:c>
-      <x:c r="F3" s="0" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="G3" s="0" t="s">
-        <x:v>35</x:v>
-      </x:c>
-      <x:c r="H3" s="0" t="s">
-        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:8">
@@ -886,25 +943,25 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>36</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>29</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="F4" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="G4" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="H4" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>41</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -921,27 +978,27 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:F4"/>
+  <x:dimension ref="A1:F6"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:6">
       <x:c r="A1" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>39</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>42</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>43</x:v>
+        <x:v>46</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:6">
@@ -949,19 +1006,19 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>44</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>45</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>46</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>47</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>48</x:v>
+        <x:v>51</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:6">
@@ -969,19 +1026,19 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>44</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="F3" s="0" t="s">
         <x:v>51</x:v>
-      </x:c>
-      <x:c r="F3" s="0" t="s">
-        <x:v>48</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:6">
@@ -989,19 +1046,59 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>44</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>52</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>54</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="F4" s="0" t="s">
-        <x:v>48</x:v>
+        <x:v>51</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:6">
+      <x:c r="A5" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="D5" s="0" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="E5" s="0" t="s">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="F5" s="0" t="s">
+        <x:v>51</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" spans="1:6">
+      <x:c r="A6" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B6" s="0" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="C6" s="0" t="s">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="D6" s="0" t="s">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="E6" s="0" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="F6" s="0" t="s">
+        <x:v>51</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1018,27 +1115,27 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:F8"/>
+  <x:dimension ref="A1:F9"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
     <x:row r="1" spans="1:6">
       <x:c r="A1" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>55</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>56</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>58</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>59</x:v>
+        <x:v>67</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:6">
@@ -1046,19 +1143,19 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>60</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>62</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>41</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:6">
@@ -1066,19 +1163,19 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>64</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>65</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>66</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>41</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:6">
@@ -1086,19 +1183,19 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>65</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="F4" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>41</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:6">
@@ -1106,19 +1203,19 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
-        <x:v>60</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="E5" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="F5" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>41</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:6">
@@ -1126,19 +1223,19 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
-        <x:v>69</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
-        <x:v>65</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="E6" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="F6" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>41</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:6">
@@ -1146,19 +1243,19 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
-        <x:v>60</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="C7" s="0" t="s">
-        <x:v>61</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="D7" s="0" t="s">
-        <x:v>68</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="E7" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="F7" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>41</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:6">
@@ -1166,19 +1263,39 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B8" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="C8" s="0" t="s">
-        <x:v>65</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="D8" s="0" t="s">
-        <x:v>70</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="E8" s="0" t="s">
-        <x:v>63</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="F8" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>41</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:6">
+      <x:c r="A9" s="0" t="s">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B9" s="0" t="s">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="C9" s="0" t="s">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="D9" s="0" t="s">
+        <x:v>79</x:v>
+      </x:c>
+      <x:c r="E9" s="0" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="F9" s="0" t="s">
+        <x:v>41</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1195,75 +1312,87 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:E4"/>
+  <x:dimension ref="A1:F4"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
-    <x:row r="1" spans="1:5">
+    <x:row r="1" spans="1:6">
       <x:c r="A1" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>72</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>73</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>22</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="2" spans="1:5">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F1" s="0" t="s">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:6">
       <x:c r="A2" s="0" t="s">
         <x:v>10</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>74</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>75</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>76</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>77</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" spans="1:5">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="F2" s="0" t="s">
+        <x:v>87</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:6">
       <x:c r="A3" s="0" t="s">
         <x:v>5</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>74</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>78</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>77</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" spans="1:5">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="F3" s="0" t="s">
+        <x:v>90</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:6">
       <x:c r="A4" s="0" t="s">
         <x:v>15</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>80</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>81</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>82</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>77</x:v>
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="F4" s="0" t="s">
+        <x:v>94</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1285,22 +1414,22 @@
   <x:sheetData>
     <x:row r="1" spans="1:6">
       <x:c r="A1" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>83</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>84</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>85</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>86</x:v>
+        <x:v>98</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:6">
@@ -1308,19 +1437,19 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>87</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>88</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>89</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>90</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>91</x:v>
+        <x:v>103</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:6">
@@ -1328,19 +1457,19 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>92</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>93</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>94</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
-        <x:v>95</x:v>
+        <x:v>107</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:6">
@@ -1348,19 +1477,19 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>96</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>93</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>64</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="F4" s="0" t="s">
-        <x:v>97</x:v>
+        <x:v>109</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:6">
@@ -1368,19 +1497,19 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
-        <x:v>98</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>99</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>60</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="E5" s="0" t="s">
-        <x:v>100</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="F5" s="0" t="s">
-        <x:v>28</x:v>
+        <x:v>31</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1402,22 +1531,22 @@
   <x:sheetData>
     <x:row r="1" spans="1:6">
       <x:c r="A1" s="0" t="s">
-        <x:v>19</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>83</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>71</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>101</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>102</x:v>
+        <x:v>114</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:6">
@@ -1425,19 +1554,19 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>103</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>104</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>105</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
-        <x:v>106</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>107</x:v>
+        <x:v>90</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:6">
@@ -1445,19 +1574,19 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>108</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>104</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>99</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
-        <x:v>109</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
-        <x:v>110</x:v>
+        <x:v>94</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:6">
@@ -1465,19 +1594,91 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>111</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>112</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>105</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>113</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="F4" s="0" t="s">
-        <x:v>114</x:v>
+        <x:v>123</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
+  <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+  <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
+  <x:headerFooter/>
+  <x:tableParts count="0"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
+  <x:sheetPr>
+    <x:outlinePr summaryBelow="1" summaryRight="1"/>
+  </x:sheetPr>
+  <x:dimension ref="A1:C5"/>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1" spans="1:3">
+      <x:c r="A1" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B1" s="0" t="s">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="C1" s="0" t="s">
+        <x:v>124</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:3">
+      <x:c r="A2" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B2" s="0" t="s">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="C2" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" spans="1:3">
+      <x:c r="A3" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B3" s="0" t="s">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="C3" s="0" t="s">
+        <x:v>125</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" spans="1:3">
+      <x:c r="A4" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B4" s="0" t="s">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="s">
+        <x:v>126</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" spans="1:3">
+      <x:c r="A5" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
+        <x:v>127</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
+        <x:v>78</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>